<commit_message>
Atualização automática portal convênios
</commit_message>
<xml_diff>
--- a/upload/pagamentorp2022.xlsx
+++ b/upload/pagamentorp2022.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q578"/>
+  <dimension ref="A1:Q577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47064,12 +47064,12 @@
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>9318850</t>
+          <t>9318851</t>
         </is>
       </c>
       <c r="B537" s="2" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>593</t>
         </is>
       </c>
       <c r="C537" s="2" t="inlineStr">
@@ -47079,12 +47079,12 @@
       </c>
       <c r="D537" s="2" t="inlineStr">
         <is>
-          <t>COMUNIDADE TERAPEUTICA CAVERNA DE ADULAO - CTCA</t>
+          <t>INSTITUTO CPL PARA DE MINAS</t>
         </is>
       </c>
       <c r="E537" s="2" t="inlineStr">
         <is>
-          <t>15.171.442/0001-78</t>
+          <t>07.604.596/0001-88</t>
         </is>
       </c>
       <c r="F537" s="2" t="inlineStr">
@@ -47104,12 +47104,12 @@
       </c>
       <c r="I537" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J537" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K537" s="2" t="inlineStr">
@@ -47119,7 +47119,7 @@
       </c>
       <c r="L537" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M537" s="2" t="inlineStr">
@@ -47134,7 +47134,7 @@
       </c>
       <c r="O537" s="2" t="inlineStr">
         <is>
-          <t>86954</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P537" s="2" t="inlineStr">
@@ -47144,49 +47144,49 @@
       </c>
       <c r="Q537" s="2" t="inlineStr">
         <is>
-          <t>86954</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>9318851</t>
+          <t>9318852</t>
         </is>
       </c>
       <c r="B538" s="2" t="inlineStr">
         <is>
-          <t>593</t>
+          <t>393</t>
         </is>
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>2021-12-30 00:00:00</t>
+          <t>2021-12-31 00:00:00</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
         <is>
-          <t>INSTITUTO CPL PARA DE MINAS</t>
+          <t>PM ERVALIA</t>
         </is>
       </c>
       <c r="E538" s="2" t="inlineStr">
         <is>
-          <t>07.604.596/0001-88</t>
+          <t>18.133.306/0001-81</t>
         </is>
       </c>
       <c r="F538" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>SEINFRA</t>
         </is>
       </c>
       <c r="G538" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="H538" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
         </is>
       </c>
       <c r="I538" s="2" t="inlineStr">
@@ -47226,7 +47226,7 @@
       </c>
       <c r="P538" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1400000</t>
         </is>
       </c>
       <c r="Q538" s="2" t="inlineStr">
@@ -47238,42 +47238,42 @@
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>9318852</t>
+          <t>9318853</t>
         </is>
       </c>
       <c r="B539" s="2" t="inlineStr">
         <is>
-          <t>393</t>
+          <t>600</t>
         </is>
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>2021-12-31 00:00:00</t>
+          <t>2021-12-30 00:00:00</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
         <is>
-          <t>PM ERVALIA</t>
+          <t>ASSOCIACAO DE PAIS E AMIGOS DOS EXCEPCIONAIS</t>
         </is>
       </c>
       <c r="E539" s="2" t="inlineStr">
         <is>
-          <t>18.133.306/0001-81</t>
+          <t>00.909.916/0001-69</t>
         </is>
       </c>
       <c r="F539" s="2" t="inlineStr">
         <is>
-          <t>SEINFRA</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G539" s="2" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H539" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I539" s="2" t="inlineStr">
@@ -47313,7 +47313,7 @@
       </c>
       <c r="P539" s="2" t="inlineStr">
         <is>
-          <t>1400000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q539" s="2" t="inlineStr">
@@ -47325,12 +47325,12 @@
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>9318853</t>
+          <t>9318854</t>
         </is>
       </c>
       <c r="B540" s="2" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>599</t>
         </is>
       </c>
       <c r="C540" s="2" t="inlineStr">
@@ -47340,12 +47340,12 @@
       </c>
       <c r="D540" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO DE PAIS E AMIGOS DOS EXCEPCIONAIS</t>
+          <t>CENTRO DE EDUCACAO INFANTIL COMUNITARIO MARIA GERALDA MARTUCHELI</t>
         </is>
       </c>
       <c r="E540" s="2" t="inlineStr">
         <is>
-          <t>00.909.916/0001-69</t>
+          <t>06.067.744/0001-00</t>
         </is>
       </c>
       <c r="F540" s="2" t="inlineStr">
@@ -47365,12 +47365,12 @@
       </c>
       <c r="I540" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J540" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K540" s="2" t="inlineStr">
@@ -47380,7 +47380,7 @@
       </c>
       <c r="L540" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M540" s="2" t="inlineStr">
@@ -47412,12 +47412,12 @@
     <row r="541">
       <c r="A541" s="2" t="inlineStr">
         <is>
-          <t>9318854</t>
+          <t>9318856</t>
         </is>
       </c>
       <c r="B541" s="2" t="inlineStr">
         <is>
-          <t>599</t>
+          <t>595</t>
         </is>
       </c>
       <c r="C541" s="2" t="inlineStr">
@@ -47427,12 +47427,12 @@
       </c>
       <c r="D541" s="2" t="inlineStr">
         <is>
-          <t>CENTRO DE EDUCACAO INFANTIL COMUNITARIO MARIA GERALDA MARTUCHELI</t>
+          <t>ASSOCIACAO DE PAIS E AMIGOS DOS EXCEPCIONAIS</t>
         </is>
       </c>
       <c r="E541" s="2" t="inlineStr">
         <is>
-          <t>06.067.744/0001-00</t>
+          <t>04.014.664/0001-60</t>
         </is>
       </c>
       <c r="F541" s="2" t="inlineStr">
@@ -47452,12 +47452,12 @@
       </c>
       <c r="I541" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J541" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K541" s="2" t="inlineStr">
@@ -47467,7 +47467,7 @@
       </c>
       <c r="L541" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M541" s="2" t="inlineStr">
@@ -47499,12 +47499,12 @@
     <row r="542">
       <c r="A542" s="2" t="inlineStr">
         <is>
-          <t>9318856</t>
+          <t>9318857</t>
         </is>
       </c>
       <c r="B542" s="2" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>597</t>
         </is>
       </c>
       <c r="C542" s="2" t="inlineStr">
@@ -47514,12 +47514,12 @@
       </c>
       <c r="D542" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO DE PAIS E AMIGOS DOS EXCEPCIONAIS</t>
+          <t>ASILO CONFRADE FRANCISCO VENANCIO PEREIRA/SAO FRANCISCO PAUL</t>
         </is>
       </c>
       <c r="E542" s="2" t="inlineStr">
         <is>
-          <t>04.014.664/0001-60</t>
+          <t>04.978.840/0001-84</t>
         </is>
       </c>
       <c r="F542" s="2" t="inlineStr">
@@ -47539,12 +47539,12 @@
       </c>
       <c r="I542" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J542" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K542" s="2" t="inlineStr">
@@ -47554,7 +47554,7 @@
       </c>
       <c r="L542" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M542" s="2" t="inlineStr">
@@ -47586,12 +47586,12 @@
     <row r="543">
       <c r="A543" s="2" t="inlineStr">
         <is>
-          <t>9318857</t>
+          <t>9318858</t>
         </is>
       </c>
       <c r="B543" s="2" t="inlineStr">
         <is>
-          <t>597</t>
+          <t>3227</t>
         </is>
       </c>
       <c r="C543" s="2" t="inlineStr">
@@ -47601,27 +47601,27 @@
       </c>
       <c r="D543" s="2" t="inlineStr">
         <is>
-          <t>ASILO CONFRADE FRANCISCO VENANCIO PEREIRA/SAO FRANCISCO PAUL</t>
+          <t>LAR DOS IDOSOS JOSE VERCOSA JUNIOR</t>
         </is>
       </c>
       <c r="E543" s="2" t="inlineStr">
         <is>
-          <t>04.978.840/0001-84</t>
+          <t>18.222.034/0001-96</t>
         </is>
       </c>
       <c r="F543" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G543" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H543" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I543" s="2" t="inlineStr">
@@ -47646,12 +47646,12 @@
       </c>
       <c r="M543" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N543" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O543" s="2" t="inlineStr">
@@ -47661,7 +47661,7 @@
       </c>
       <c r="P543" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>20128</t>
         </is>
       </c>
       <c r="Q543" s="2" t="inlineStr">
@@ -47678,7 +47678,7 @@
       </c>
       <c r="B544" s="2" t="inlineStr">
         <is>
-          <t>3227</t>
+          <t>3228</t>
         </is>
       </c>
       <c r="C544" s="2" t="inlineStr">
@@ -47713,12 +47713,12 @@
       </c>
       <c r="I544" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J544" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K544" s="2" t="inlineStr">
@@ -47728,7 +47728,7 @@
       </c>
       <c r="L544" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M544" s="2" t="inlineStr">
@@ -47748,7 +47748,7 @@
       </c>
       <c r="P544" s="2" t="inlineStr">
         <is>
-          <t>20128</t>
+          <t>92860</t>
         </is>
       </c>
       <c r="Q544" s="2" t="inlineStr">
@@ -47760,42 +47760,42 @@
     <row r="545">
       <c r="A545" s="2" t="inlineStr">
         <is>
-          <t>9318858</t>
+          <t>9318859</t>
         </is>
       </c>
       <c r="B545" s="2" t="inlineStr">
         <is>
-          <t>3228</t>
+          <t>397</t>
         </is>
       </c>
       <c r="C545" s="2" t="inlineStr">
         <is>
-          <t>2021-12-30 00:00:00</t>
+          <t>2021-12-31 00:00:00</t>
         </is>
       </c>
       <c r="D545" s="2" t="inlineStr">
         <is>
-          <t>LAR DOS IDOSOS JOSE VERCOSA JUNIOR</t>
+          <t>PM ARAPORA</t>
         </is>
       </c>
       <c r="E545" s="2" t="inlineStr">
         <is>
-          <t>18.222.034/0001-96</t>
+          <t>23.098.510/0001-49</t>
         </is>
       </c>
       <c r="F545" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEINFRA</t>
         </is>
       </c>
       <c r="G545" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="H545" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
         </is>
       </c>
       <c r="I545" s="2" t="inlineStr">
@@ -47820,12 +47820,12 @@
       </c>
       <c r="M545" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N545" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O545" s="2" t="inlineStr">
@@ -47835,7 +47835,7 @@
       </c>
       <c r="P545" s="2" t="inlineStr">
         <is>
-          <t>92860</t>
+          <t>200000</t>
         </is>
       </c>
       <c r="Q545" s="2" t="inlineStr">
@@ -47847,52 +47847,52 @@
     <row r="546">
       <c r="A546" s="2" t="inlineStr">
         <is>
-          <t>9318859</t>
+          <t>9318860</t>
         </is>
       </c>
       <c r="B546" s="2" t="inlineStr">
         <is>
-          <t>397</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C546" s="2" t="inlineStr">
         <is>
-          <t>2021-12-31 00:00:00</t>
+          <t>2021-12-30 00:00:00</t>
         </is>
       </c>
       <c r="D546" s="2" t="inlineStr">
         <is>
-          <t>PM ARAPORA</t>
+          <t>GRUPO EDUCACAO, ETICA E CIDADANIA</t>
         </is>
       </c>
       <c r="E546" s="2" t="inlineStr">
         <is>
-          <t>23.098.510/0001-49</t>
+          <t>05.543.739/0001-63</t>
         </is>
       </c>
       <c r="F546" s="2" t="inlineStr">
         <is>
-          <t>SEINFRA</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G546" s="2" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H546" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I546" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J546" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K546" s="2" t="inlineStr">
@@ -47902,7 +47902,7 @@
       </c>
       <c r="L546" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M546" s="2" t="inlineStr">
@@ -47917,29 +47917,29 @@
       </c>
       <c r="O546" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>78500</t>
         </is>
       </c>
       <c r="P546" s="2" t="inlineStr">
         <is>
-          <t>200000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q546" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>78500</t>
         </is>
       </c>
     </row>
     <row r="547">
       <c r="A547" s="2" t="inlineStr">
         <is>
-          <t>9318860</t>
+          <t>9318861</t>
         </is>
       </c>
       <c r="B547" s="2" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>601</t>
         </is>
       </c>
       <c r="C547" s="2" t="inlineStr">
@@ -47949,12 +47949,12 @@
       </c>
       <c r="D547" s="2" t="inlineStr">
         <is>
-          <t>GRUPO EDUCACAO, ETICA E CIDADANIA</t>
+          <t>CENTRO DE CONVIVENCIA PARA IDOSOS PADRE JOSE GERALDO DAS MERCES</t>
         </is>
       </c>
       <c r="E547" s="2" t="inlineStr">
         <is>
-          <t>05.543.739/0001-63</t>
+          <t>03.437.717/0001-93</t>
         </is>
       </c>
       <c r="F547" s="2" t="inlineStr">
@@ -48004,7 +48004,7 @@
       </c>
       <c r="O547" s="2" t="inlineStr">
         <is>
-          <t>78500</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P547" s="2" t="inlineStr">
@@ -48014,19 +48014,19 @@
       </c>
       <c r="Q547" s="2" t="inlineStr">
         <is>
-          <t>78500</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="548">
       <c r="A548" s="2" t="inlineStr">
         <is>
-          <t>9318861</t>
+          <t>9318862</t>
         </is>
       </c>
       <c r="B548" s="2" t="inlineStr">
         <is>
-          <t>601</t>
+          <t>3223</t>
         </is>
       </c>
       <c r="C548" s="2" t="inlineStr">
@@ -48036,27 +48036,27 @@
       </c>
       <c r="D548" s="2" t="inlineStr">
         <is>
-          <t>CENTRO DE CONVIVENCIA PARA IDOSOS PADRE JOSE GERALDO DAS MERCES</t>
+          <t>ASSOCIACAO FREI INOCENCIO</t>
         </is>
       </c>
       <c r="E548" s="2" t="inlineStr">
         <is>
-          <t>03.437.717/0001-93</t>
+          <t>07.715.739/0001-29</t>
         </is>
       </c>
       <c r="F548" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G548" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H548" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I548" s="2" t="inlineStr">
@@ -48081,12 +48081,12 @@
       </c>
       <c r="M548" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N548" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O548" s="2" t="inlineStr">
@@ -48096,7 +48096,7 @@
       </c>
       <c r="P548" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114986.52</t>
         </is>
       </c>
       <c r="Q548" s="2" t="inlineStr">
@@ -48108,52 +48108,52 @@
     <row r="549">
       <c r="A549" s="2" t="inlineStr">
         <is>
-          <t>9318862</t>
+          <t>9318863</t>
         </is>
       </c>
       <c r="B549" s="2" t="inlineStr">
         <is>
-          <t>3223</t>
+          <t>392</t>
         </is>
       </c>
       <c r="C549" s="2" t="inlineStr">
         <is>
-          <t>2021-12-30 00:00:00</t>
+          <t>2021-12-31 00:00:00</t>
         </is>
       </c>
       <c r="D549" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO FREI INOCENCIO</t>
+          <t>PM SANTA MARIA DE ITABIRA</t>
         </is>
       </c>
       <c r="E549" s="2" t="inlineStr">
         <is>
-          <t>07.715.739/0001-29</t>
+          <t>18.299.453/0001-26</t>
         </is>
       </c>
       <c r="F549" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEINFRA</t>
         </is>
       </c>
       <c r="G549" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="H549" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
         </is>
       </c>
       <c r="I549" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J549" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K549" s="2" t="inlineStr">
@@ -48163,17 +48163,17 @@
       </c>
       <c r="L549" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M549" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N549" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O549" s="2" t="inlineStr">
@@ -48183,7 +48183,7 @@
       </c>
       <c r="P549" s="2" t="inlineStr">
         <is>
-          <t>114986.52</t>
+          <t>150000</t>
         </is>
       </c>
       <c r="Q549" s="2" t="inlineStr">
@@ -48195,42 +48195,42 @@
     <row r="550">
       <c r="A550" s="2" t="inlineStr">
         <is>
-          <t>9318863</t>
+          <t>9318864</t>
         </is>
       </c>
       <c r="B550" s="2" t="inlineStr">
         <is>
-          <t>392</t>
+          <t>602</t>
         </is>
       </c>
       <c r="C550" s="2" t="inlineStr">
         <is>
-          <t>2021-12-31 00:00:00</t>
+          <t>2021-12-30 00:00:00</t>
         </is>
       </c>
       <c r="D550" s="2" t="inlineStr">
         <is>
-          <t>PM SANTA MARIA DE ITABIRA</t>
+          <t>SASFRA SERVICO ASSISTENCIAL SALAO DO ENCONTRO</t>
         </is>
       </c>
       <c r="E550" s="2" t="inlineStr">
         <is>
-          <t>18.299.453/0001-26</t>
+          <t>16.701.872/0001-17</t>
         </is>
       </c>
       <c r="F550" s="2" t="inlineStr">
         <is>
-          <t>SEINFRA</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G550" s="2" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H550" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I550" s="2" t="inlineStr">
@@ -48270,7 +48270,7 @@
       </c>
       <c r="P550" s="2" t="inlineStr">
         <is>
-          <t>150000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q550" s="2" t="inlineStr">
@@ -48282,12 +48282,12 @@
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
         <is>
-          <t>9318864</t>
+          <t>9318865</t>
         </is>
       </c>
       <c r="B551" s="2" t="inlineStr">
         <is>
-          <t>602</t>
+          <t>603</t>
         </is>
       </c>
       <c r="C551" s="2" t="inlineStr">
@@ -48297,12 +48297,12 @@
       </c>
       <c r="D551" s="2" t="inlineStr">
         <is>
-          <t>SASFRA SERVICO ASSISTENCIAL SALAO DO ENCONTRO</t>
+          <t>ASSOCIACAO COMUNITARIA DO DIST DE SANTANA DO CAPIVARI</t>
         </is>
       </c>
       <c r="E551" s="2" t="inlineStr">
         <is>
-          <t>16.701.872/0001-17</t>
+          <t>19.089.853/0001-70</t>
         </is>
       </c>
       <c r="F551" s="2" t="inlineStr">
@@ -48369,42 +48369,42 @@
     <row r="552">
       <c r="A552" s="2" t="inlineStr">
         <is>
-          <t>9318865</t>
+          <t>9318866</t>
         </is>
       </c>
       <c r="B552" s="2" t="inlineStr">
         <is>
-          <t>603</t>
+          <t>398</t>
         </is>
       </c>
       <c r="C552" s="2" t="inlineStr">
         <is>
-          <t>2021-12-30 00:00:00</t>
+          <t>2021-12-31 00:00:00</t>
         </is>
       </c>
       <c r="D552" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO COMUNITARIA DO DIST DE SANTANA DO CAPIVARI</t>
+          <t>PM SENADOR CORTES</t>
         </is>
       </c>
       <c r="E552" s="2" t="inlineStr">
         <is>
-          <t>19.089.853/0001-70</t>
+          <t>17.724.576/0001-02</t>
         </is>
       </c>
       <c r="F552" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>SEINFRA</t>
         </is>
       </c>
       <c r="G552" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="H552" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
         </is>
       </c>
       <c r="I552" s="2" t="inlineStr">
@@ -48444,7 +48444,7 @@
       </c>
       <c r="P552" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>149999</t>
         </is>
       </c>
       <c r="Q552" s="2" t="inlineStr">
@@ -48456,52 +48456,52 @@
     <row r="553">
       <c r="A553" s="2" t="inlineStr">
         <is>
-          <t>9318866</t>
+          <t>9318867</t>
         </is>
       </c>
       <c r="B553" s="2" t="inlineStr">
         <is>
-          <t>398</t>
+          <t>3224</t>
         </is>
       </c>
       <c r="C553" s="2" t="inlineStr">
         <is>
-          <t>2021-12-31 00:00:00</t>
+          <t>2021-12-30 00:00:00</t>
         </is>
       </c>
       <c r="D553" s="2" t="inlineStr">
         <is>
-          <t>PM SENADOR CORTES</t>
+          <t>INSTITUTO DE ACOLHIMENTO CASA DO CAMINHO</t>
         </is>
       </c>
       <c r="E553" s="2" t="inlineStr">
         <is>
-          <t>17.724.576/0001-02</t>
+          <t>29.937.767/0001-23</t>
         </is>
       </c>
       <c r="F553" s="2" t="inlineStr">
         <is>
-          <t>SEINFRA</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G553" s="2" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H553" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I553" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J553" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K553" s="2" t="inlineStr">
@@ -48511,44 +48511,44 @@
       </c>
       <c r="L553" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M553" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>71</t>
         </is>
       </c>
       <c r="N553" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
         </is>
       </c>
       <c r="O553" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114246</t>
         </is>
       </c>
       <c r="P553" s="2" t="inlineStr">
         <is>
-          <t>149999</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q553" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114246</t>
         </is>
       </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">
         <is>
-          <t>9318867</t>
+          <t>9318868</t>
         </is>
       </c>
       <c r="B554" s="2" t="inlineStr">
         <is>
-          <t>3224</t>
+          <t>3213</t>
         </is>
       </c>
       <c r="C554" s="2" t="inlineStr">
@@ -48558,12 +48558,12 @@
       </c>
       <c r="D554" s="2" t="inlineStr">
         <is>
-          <t>INSTITUTO DE ACOLHIMENTO CASA DO CAMINHO</t>
+          <t>ASSOCIACAO COM.DO MOVIMENTO FAMILIAR CRISTAO DE AIURUOCA</t>
         </is>
       </c>
       <c r="E554" s="2" t="inlineStr">
         <is>
-          <t>29.937.767/0001-23</t>
+          <t>19.090.034/0001-42</t>
         </is>
       </c>
       <c r="F554" s="2" t="inlineStr">
@@ -48603,39 +48603,39 @@
       </c>
       <c r="M554" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N554" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O554" s="2" t="inlineStr">
         <is>
-          <t>114246</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P554" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>114997.7</t>
         </is>
       </c>
       <c r="Q554" s="2" t="inlineStr">
         <is>
-          <t>114246</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">
         <is>
-          <t>9318868</t>
+          <t>9318869</t>
         </is>
       </c>
       <c r="B555" s="2" t="inlineStr">
         <is>
-          <t>3213</t>
+          <t>3222</t>
         </is>
       </c>
       <c r="C555" s="2" t="inlineStr">
@@ -48645,12 +48645,12 @@
       </c>
       <c r="D555" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO COM.DO MOVIMENTO FAMILIAR CRISTAO DE AIURUOCA</t>
+          <t>ABRIGO INSTITUCIONAL NOSSO LAR</t>
         </is>
       </c>
       <c r="E555" s="2" t="inlineStr">
         <is>
-          <t>19.090.034/0001-42</t>
+          <t>04.868.943/0001-91</t>
         </is>
       </c>
       <c r="F555" s="2" t="inlineStr">
@@ -48690,27 +48690,27 @@
       </c>
       <c r="M555" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>71</t>
         </is>
       </c>
       <c r="N555" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
         </is>
       </c>
       <c r="O555" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110740</t>
         </is>
       </c>
       <c r="P555" s="2" t="inlineStr">
         <is>
-          <t>114997.7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q555" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>110740</t>
         </is>
       </c>
     </row>
@@ -48722,7 +48722,7 @@
       </c>
       <c r="B556" s="2" t="inlineStr">
         <is>
-          <t>3222</t>
+          <t>3233</t>
         </is>
       </c>
       <c r="C556" s="2" t="inlineStr">
@@ -48757,12 +48757,12 @@
       </c>
       <c r="I556" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J556" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K556" s="2" t="inlineStr">
@@ -48772,7 +48772,7 @@
       </c>
       <c r="L556" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M556" s="2" t="inlineStr">
@@ -48787,59 +48787,59 @@
       </c>
       <c r="O556" s="2" t="inlineStr">
         <is>
-          <t>110740</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P556" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1082.66</t>
         </is>
       </c>
       <c r="Q556" s="2" t="inlineStr">
         <is>
-          <t>110740</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="557">
       <c r="A557" s="2" t="inlineStr">
         <is>
-          <t>9318869</t>
+          <t>9318870</t>
         </is>
       </c>
       <c r="B557" s="2" t="inlineStr">
         <is>
-          <t>3233</t>
+          <t>401</t>
         </is>
       </c>
       <c r="C557" s="2" t="inlineStr">
         <is>
-          <t>2021-12-30 00:00:00</t>
+          <t>2021-12-31 00:00:00</t>
         </is>
       </c>
       <c r="D557" s="2" t="inlineStr">
         <is>
-          <t>ABRIGO INSTITUCIONAL NOSSO LAR</t>
+          <t>PM MONTE ALEGRE DE MINAS</t>
         </is>
       </c>
       <c r="E557" s="2" t="inlineStr">
         <is>
-          <t>04.868.943/0001-91</t>
+          <t>18.431.155/0001-48</t>
         </is>
       </c>
       <c r="F557" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEINFRA</t>
         </is>
       </c>
       <c r="G557" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1301</t>
         </is>
       </c>
       <c r="H557" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
         </is>
       </c>
       <c r="I557" s="2" t="inlineStr">
@@ -48864,12 +48864,12 @@
       </c>
       <c r="M557" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N557" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O557" s="2" t="inlineStr">
@@ -48879,7 +48879,7 @@
       </c>
       <c r="P557" s="2" t="inlineStr">
         <is>
-          <t>1082.66</t>
+          <t>200000</t>
         </is>
       </c>
       <c r="Q557" s="2" t="inlineStr">
@@ -48891,42 +48891,42 @@
     <row r="558">
       <c r="A558" s="2" t="inlineStr">
         <is>
-          <t>9318870</t>
+          <t>9318871</t>
         </is>
       </c>
       <c r="B558" s="2" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>604</t>
         </is>
       </c>
       <c r="C558" s="2" t="inlineStr">
         <is>
-          <t>2021-12-31 00:00:00</t>
+          <t>2021-12-30 00:00:00</t>
         </is>
       </c>
       <c r="D558" s="2" t="inlineStr">
         <is>
-          <t>PM MONTE ALEGRE DE MINAS</t>
+          <t>INST PADRE ANTONIO FERREIRA MARTINS-CENTRO DE ACAO SOCIAL E CIDADANIA</t>
         </is>
       </c>
       <c r="E558" s="2" t="inlineStr">
         <is>
-          <t>18.431.155/0001-48</t>
+          <t>08.576.487/0001-67</t>
         </is>
       </c>
       <c r="F558" s="2" t="inlineStr">
         <is>
-          <t>SEINFRA</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G558" s="2" t="inlineStr">
         <is>
-          <t>1301</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H558" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA E MOBILIDADE</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I558" s="2" t="inlineStr">
@@ -48966,7 +48966,7 @@
       </c>
       <c r="P558" s="2" t="inlineStr">
         <is>
-          <t>200000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q558" s="2" t="inlineStr">
@@ -48978,12 +48978,12 @@
     <row r="559">
       <c r="A559" s="2" t="inlineStr">
         <is>
-          <t>9318871</t>
+          <t>9318872</t>
         </is>
       </c>
       <c r="B559" s="2" t="inlineStr">
         <is>
-          <t>604</t>
+          <t>3221</t>
         </is>
       </c>
       <c r="C559" s="2" t="inlineStr">
@@ -48993,27 +48993,27 @@
       </c>
       <c r="D559" s="2" t="inlineStr">
         <is>
-          <t>INST PADRE ANTONIO FERREIRA MARTINS-CENTRO DE ACAO SOCIAL E CIDADANIA</t>
+          <t>ASSOCIACAO JOAO PAULO II</t>
         </is>
       </c>
       <c r="E559" s="2" t="inlineStr">
         <is>
-          <t>08.576.487/0001-67</t>
+          <t>08.027.860/0001-20</t>
         </is>
       </c>
       <c r="F559" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G559" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H559" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I559" s="2" t="inlineStr">
@@ -49038,12 +49038,12 @@
       </c>
       <c r="M559" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N559" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O559" s="2" t="inlineStr">
@@ -49053,7 +49053,7 @@
       </c>
       <c r="P559" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>115000</t>
         </is>
       </c>
       <c r="Q559" s="2" t="inlineStr">
@@ -49065,12 +49065,12 @@
     <row r="560">
       <c r="A560" s="2" t="inlineStr">
         <is>
-          <t>9318872</t>
+          <t>9318874</t>
         </is>
       </c>
       <c r="B560" s="2" t="inlineStr">
         <is>
-          <t>3221</t>
+          <t>3214</t>
         </is>
       </c>
       <c r="C560" s="2" t="inlineStr">
@@ -49080,12 +49080,12 @@
       </c>
       <c r="D560" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO JOAO PAULO II</t>
+          <t>ASILO SAO VICENTE DE PAULO DE POCRANE</t>
         </is>
       </c>
       <c r="E560" s="2" t="inlineStr">
         <is>
-          <t>08.027.860/0001-20</t>
+          <t>03.165.540/0001-13</t>
         </is>
       </c>
       <c r="F560" s="2" t="inlineStr">
@@ -49105,12 +49105,12 @@
       </c>
       <c r="I560" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J560" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K560" s="2" t="inlineStr">
@@ -49120,32 +49120,32 @@
       </c>
       <c r="L560" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M560" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>71</t>
         </is>
       </c>
       <c r="N560" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
         </is>
       </c>
       <c r="O560" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12715.45</t>
         </is>
       </c>
       <c r="P560" s="2" t="inlineStr">
         <is>
-          <t>115000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q560" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12715.45</t>
         </is>
       </c>
     </row>
@@ -49157,7 +49157,7 @@
       </c>
       <c r="B561" s="2" t="inlineStr">
         <is>
-          <t>3214</t>
+          <t>3215</t>
         </is>
       </c>
       <c r="C561" s="2" t="inlineStr">
@@ -49192,12 +49192,12 @@
       </c>
       <c r="I561" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J561" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K561" s="2" t="inlineStr">
@@ -49207,7 +49207,7 @@
       </c>
       <c r="L561" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M561" s="2" t="inlineStr">
@@ -49222,7 +49222,7 @@
       </c>
       <c r="O561" s="2" t="inlineStr">
         <is>
-          <t>12715.45</t>
+          <t>100284.1</t>
         </is>
       </c>
       <c r="P561" s="2" t="inlineStr">
@@ -49232,19 +49232,19 @@
       </c>
       <c r="Q561" s="2" t="inlineStr">
         <is>
-          <t>12715.45</t>
+          <t>100284.1</t>
         </is>
       </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
         <is>
-          <t>9318874</t>
+          <t>9318875</t>
         </is>
       </c>
       <c r="B562" s="2" t="inlineStr">
         <is>
-          <t>3215</t>
+          <t>607</t>
         </is>
       </c>
       <c r="C562" s="2" t="inlineStr">
@@ -49254,27 +49254,27 @@
       </c>
       <c r="D562" s="2" t="inlineStr">
         <is>
-          <t>ASILO SAO VICENTE DE PAULO DE POCRANE</t>
+          <t>ASSOCIACAO ACONCHEGO - LAR PARA IDOSOS</t>
         </is>
       </c>
       <c r="E562" s="2" t="inlineStr">
         <is>
-          <t>03.165.540/0001-13</t>
+          <t>30.276.755/0001-84</t>
         </is>
       </c>
       <c r="F562" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G562" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H562" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I562" s="2" t="inlineStr">
@@ -49299,17 +49299,17 @@
       </c>
       <c r="M562" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N562" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O562" s="2" t="inlineStr">
         <is>
-          <t>100284.1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P562" s="2" t="inlineStr">
@@ -49319,19 +49319,19 @@
       </c>
       <c r="Q562" s="2" t="inlineStr">
         <is>
-          <t>100284.1</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
         <is>
-          <t>9318875</t>
+          <t>9318876</t>
         </is>
       </c>
       <c r="B563" s="2" t="inlineStr">
         <is>
-          <t>607</t>
+          <t>605</t>
         </is>
       </c>
       <c r="C563" s="2" t="inlineStr">
@@ -49341,12 +49341,12 @@
       </c>
       <c r="D563" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO ACONCHEGO - LAR PARA IDOSOS</t>
+          <t>ASSOCIACAO DO PEQUENO CRISTO</t>
         </is>
       </c>
       <c r="E563" s="2" t="inlineStr">
         <is>
-          <t>30.276.755/0001-84</t>
+          <t>42.783.621/0001-39</t>
         </is>
       </c>
       <c r="F563" s="2" t="inlineStr">
@@ -49413,12 +49413,12 @@
     <row r="564">
       <c r="A564" s="2" t="inlineStr">
         <is>
-          <t>9318876</t>
+          <t>9318877</t>
         </is>
       </c>
       <c r="B564" s="2" t="inlineStr">
         <is>
-          <t>605</t>
+          <t>606</t>
         </is>
       </c>
       <c r="C564" s="2" t="inlineStr">
@@ -49428,12 +49428,12 @@
       </c>
       <c r="D564" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO DO PEQUENO CRISTO</t>
+          <t>ARUR-ASSOCIACAO DOS REUMATICOS DE UBERLANDIA E REGIAO</t>
         </is>
       </c>
       <c r="E564" s="2" t="inlineStr">
         <is>
-          <t>42.783.621/0001-39</t>
+          <t>01.411.315/0001-94</t>
         </is>
       </c>
       <c r="F564" s="2" t="inlineStr">
@@ -49500,12 +49500,12 @@
     <row r="565">
       <c r="A565" s="2" t="inlineStr">
         <is>
-          <t>9318877</t>
+          <t>9318878</t>
         </is>
       </c>
       <c r="B565" s="2" t="inlineStr">
         <is>
-          <t>606</t>
+          <t>610</t>
         </is>
       </c>
       <c r="C565" s="2" t="inlineStr">
@@ -49515,12 +49515,12 @@
       </c>
       <c r="D565" s="2" t="inlineStr">
         <is>
-          <t>ARUR-ASSOCIACAO DOS REUMATICOS DE UBERLANDIA E REGIAO</t>
+          <t>PM RUBELITA</t>
         </is>
       </c>
       <c r="E565" s="2" t="inlineStr">
         <is>
-          <t>01.411.315/0001-94</t>
+          <t>24.363.590/0001-85</t>
         </is>
       </c>
       <c r="F565" s="2" t="inlineStr">
@@ -49570,7 +49570,7 @@
       </c>
       <c r="O565" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>50000</t>
         </is>
       </c>
       <c r="P565" s="2" t="inlineStr">
@@ -49580,19 +49580,19 @@
       </c>
       <c r="Q565" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>50000</t>
         </is>
       </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">
         <is>
-          <t>9318878</t>
+          <t>9318881</t>
         </is>
       </c>
       <c r="B566" s="2" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>608</t>
         </is>
       </c>
       <c r="C566" s="2" t="inlineStr">
@@ -49602,12 +49602,12 @@
       </c>
       <c r="D566" s="2" t="inlineStr">
         <is>
-          <t>PM RUBELITA</t>
+          <t>LAR SAO VICENTE DE PAULO</t>
         </is>
       </c>
       <c r="E566" s="2" t="inlineStr">
         <is>
-          <t>24.363.590/0001-85</t>
+          <t>19.626.191/0001-20</t>
         </is>
       </c>
       <c r="F566" s="2" t="inlineStr">
@@ -49627,12 +49627,12 @@
       </c>
       <c r="I566" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J566" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K566" s="2" t="inlineStr">
@@ -49642,7 +49642,7 @@
       </c>
       <c r="L566" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M566" s="2" t="inlineStr">
@@ -49657,7 +49657,7 @@
       </c>
       <c r="O566" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P566" s="2" t="inlineStr">
@@ -49667,19 +49667,19 @@
       </c>
       <c r="Q566" s="2" t="inlineStr">
         <is>
-          <t>50000</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">
         <is>
-          <t>9318881</t>
+          <t>9318882</t>
         </is>
       </c>
       <c r="B567" s="2" t="inlineStr">
         <is>
-          <t>608</t>
+          <t>609</t>
         </is>
       </c>
       <c r="C567" s="2" t="inlineStr">
@@ -49689,12 +49689,12 @@
       </c>
       <c r="D567" s="2" t="inlineStr">
         <is>
-          <t>LAR SAO VICENTE DE PAULO</t>
+          <t>ASSOCIACAO ASSISTENCIAL CANTINA D.BERNADETE LEMOS</t>
         </is>
       </c>
       <c r="E567" s="2" t="inlineStr">
         <is>
-          <t>19.626.191/0001-20</t>
+          <t>00.973.124/0001-53</t>
         </is>
       </c>
       <c r="F567" s="2" t="inlineStr">
@@ -49761,12 +49761,12 @@
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
         <is>
-          <t>9318882</t>
+          <t>9318883</t>
         </is>
       </c>
       <c r="B568" s="2" t="inlineStr">
         <is>
-          <t>609</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C568" s="2" t="inlineStr">
@@ -49776,37 +49776,37 @@
       </c>
       <c r="D568" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO ASSISTENCIAL CANTINA D.BERNADETE LEMOS</t>
+          <t>PM ANGELANDIA</t>
         </is>
       </c>
       <c r="E568" s="2" t="inlineStr">
         <is>
-          <t>00.973.124/0001-53</t>
+          <t>01.113.937/0001-36</t>
         </is>
       </c>
       <c r="F568" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>FEI</t>
         </is>
       </c>
       <c r="G568" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>4601</t>
         </is>
       </c>
       <c r="H568" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>FUNDO ESTADUAL DOS DIREITOS DO IDOSO</t>
         </is>
       </c>
       <c r="I568" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>41</t>
         </is>
       </c>
       <c r="J568" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>CONTRIBUICOES</t>
         </is>
       </c>
       <c r="K568" s="2" t="inlineStr">
@@ -49816,22 +49816,22 @@
       </c>
       <c r="L568" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>CONTRIBUICOES</t>
         </is>
       </c>
       <c r="M568" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>45</t>
         </is>
       </c>
       <c r="N568" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>DOACOES DE PESSOAS, DE INSTITUICOES PRIVADAS OU DO EXTERIOR A ORGAO E ENTIDADES DO ESTADO</t>
         </is>
       </c>
       <c r="O568" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="P568" s="2" t="inlineStr">
@@ -49841,19 +49841,19 @@
       </c>
       <c r="Q568" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>40000</t>
         </is>
       </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
         <is>
-          <t>9318883</t>
+          <t>9318884</t>
         </is>
       </c>
       <c r="B569" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>3229</t>
         </is>
       </c>
       <c r="C569" s="2" t="inlineStr">
@@ -49863,37 +49863,37 @@
       </c>
       <c r="D569" s="2" t="inlineStr">
         <is>
-          <t>PM ANGELANDIA</t>
+          <t>CONS.PARTI.DA SOC.SAO VICENTE DE PAULO</t>
         </is>
       </c>
       <c r="E569" s="2" t="inlineStr">
         <is>
-          <t>01.113.937/0001-36</t>
+          <t>24.665.630/0001-43</t>
         </is>
       </c>
       <c r="F569" s="2" t="inlineStr">
         <is>
-          <t>FEI</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G569" s="2" t="inlineStr">
         <is>
-          <t>4601</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H569" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DOS DIREITOS DO IDOSO</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I569" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J569" s="2" t="inlineStr">
         <is>
-          <t>CONTRIBUICOES</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K569" s="2" t="inlineStr">
@@ -49903,32 +49903,32 @@
       </c>
       <c r="L569" s="2" t="inlineStr">
         <is>
-          <t>CONTRIBUICOES</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M569" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>71</t>
         </is>
       </c>
       <c r="N569" s="2" t="inlineStr">
         <is>
-          <t>DOACOES DE PESSOAS, DE INSTITUICOES PRIVADAS OU DO EXTERIOR A ORGAO E ENTIDADES DO ESTADO</t>
+          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
         </is>
       </c>
       <c r="O569" s="2" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P569" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>34066.5</t>
         </is>
       </c>
       <c r="Q569" s="2" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -49940,7 +49940,7 @@
       </c>
       <c r="B570" s="2" t="inlineStr">
         <is>
-          <t>3229</t>
+          <t>3230</t>
         </is>
       </c>
       <c r="C570" s="2" t="inlineStr">
@@ -49975,12 +49975,12 @@
       </c>
       <c r="I570" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J570" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K570" s="2" t="inlineStr">
@@ -49990,7 +49990,7 @@
       </c>
       <c r="L570" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M570" s="2" t="inlineStr">
@@ -50010,7 +50010,7 @@
       </c>
       <c r="P570" s="2" t="inlineStr">
         <is>
-          <t>34066.5</t>
+          <t>80918.34</t>
         </is>
       </c>
       <c r="Q570" s="2" t="inlineStr">
@@ -50022,12 +50022,12 @@
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
         <is>
-          <t>9318884</t>
+          <t>9318885</t>
         </is>
       </c>
       <c r="B571" s="2" t="inlineStr">
         <is>
-          <t>3230</t>
+          <t>126</t>
         </is>
       </c>
       <c r="C571" s="2" t="inlineStr">
@@ -50037,37 +50037,37 @@
       </c>
       <c r="D571" s="2" t="inlineStr">
         <is>
-          <t>CONS.PARTI.DA SOC.SAO VICENTE DE PAULO</t>
+          <t>ASSOCIACAO COMUNIDADE NOVA CRIATURA</t>
         </is>
       </c>
       <c r="E571" s="2" t="inlineStr">
         <is>
-          <t>24.665.630/0001-43</t>
+          <t>11.088.620/0001-40</t>
         </is>
       </c>
       <c r="F571" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G571" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H571" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I571" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J571" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K571" s="2" t="inlineStr">
@@ -50077,44 +50077,44 @@
       </c>
       <c r="L571" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M571" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N571" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DO FUNDO ESTADUAL DE ERRADICACAO DA MISERIA</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O571" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86954</t>
         </is>
       </c>
       <c r="P571" s="2" t="inlineStr">
         <is>
-          <t>80918.34</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Q571" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86954</t>
         </is>
       </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">
         <is>
-          <t>9318885</t>
+          <t>9318887</t>
         </is>
       </c>
       <c r="B572" s="2" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>611</t>
         </is>
       </c>
       <c r="C572" s="2" t="inlineStr">
@@ -50124,12 +50124,12 @@
       </c>
       <c r="D572" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO COMUNIDADE NOVA CRIATURA</t>
+          <t>ASSOCIACAO DE PAIS AMIGOS EXCEPCIONAIS/CARMOPOLIS DE MINAS</t>
         </is>
       </c>
       <c r="E572" s="2" t="inlineStr">
         <is>
-          <t>11.088.620/0001-40</t>
+          <t>00.809.356/0001-70</t>
         </is>
       </c>
       <c r="F572" s="2" t="inlineStr">
@@ -50149,12 +50149,12 @@
       </c>
       <c r="I572" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="J572" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="K572" s="2" t="inlineStr">
@@ -50164,7 +50164,7 @@
       </c>
       <c r="L572" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>AUXILIOS</t>
         </is>
       </c>
       <c r="M572" s="2" t="inlineStr">
@@ -50179,7 +50179,7 @@
       </c>
       <c r="O572" s="2" t="inlineStr">
         <is>
-          <t>86954</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P572" s="2" t="inlineStr">
@@ -50189,19 +50189,19 @@
       </c>
       <c r="Q572" s="2" t="inlineStr">
         <is>
-          <t>86954</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
         <is>
-          <t>9318887</t>
+          <t>9318888</t>
         </is>
       </c>
       <c r="B573" s="2" t="inlineStr">
         <is>
-          <t>611</t>
+          <t>125</t>
         </is>
       </c>
       <c r="C573" s="2" t="inlineStr">
@@ -50211,12 +50211,12 @@
       </c>
       <c r="D573" s="2" t="inlineStr">
         <is>
-          <t>ASSOCIACAO DE PAIS AMIGOS EXCEPCIONAIS/CARMOPOLIS DE MINAS</t>
+          <t>CENTRO DE RESTAURACAO VIDA NOVA</t>
         </is>
       </c>
       <c r="E573" s="2" t="inlineStr">
         <is>
-          <t>00.809.356/0001-70</t>
+          <t>09.219.152/0001-54</t>
         </is>
       </c>
       <c r="F573" s="2" t="inlineStr">
@@ -50236,12 +50236,12 @@
       </c>
       <c r="I573" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J573" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K573" s="2" t="inlineStr">
@@ -50251,7 +50251,7 @@
       </c>
       <c r="L573" s="2" t="inlineStr">
         <is>
-          <t>AUXILIOS</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M573" s="2" t="inlineStr">
@@ -50266,7 +50266,7 @@
       </c>
       <c r="O573" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86891.76</t>
         </is>
       </c>
       <c r="P573" s="2" t="inlineStr">
@@ -50276,19 +50276,19 @@
       </c>
       <c r="Q573" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>86891.76</t>
         </is>
       </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
         <is>
-          <t>9318888</t>
+          <t>9318889</t>
         </is>
       </c>
       <c r="B574" s="2" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>3232</t>
         </is>
       </c>
       <c r="C574" s="2" t="inlineStr">
@@ -50298,27 +50298,27 @@
       </c>
       <c r="D574" s="2" t="inlineStr">
         <is>
-          <t>CENTRO DE RESTAURACAO VIDA NOVA</t>
+          <t>CASA ESPIRITA DO SAMARITANO</t>
         </is>
       </c>
       <c r="E574" s="2" t="inlineStr">
         <is>
-          <t>09.219.152/0001-54</t>
+          <t>01.320.148/0001-76</t>
         </is>
       </c>
       <c r="F574" s="2" t="inlineStr">
         <is>
-          <t>SEDESE</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G574" s="2" t="inlineStr">
         <is>
-          <t>1481</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H574" s="2" t="inlineStr">
         <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I574" s="2" t="inlineStr">
@@ -50343,17 +50343,17 @@
       </c>
       <c r="M574" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N574" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS ORDINARIOS</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O574" s="2" t="inlineStr">
         <is>
-          <t>86891.76</t>
+          <t>114235</t>
         </is>
       </c>
       <c r="P574" s="2" t="inlineStr">
@@ -50363,19 +50363,19 @@
       </c>
       <c r="Q574" s="2" t="inlineStr">
         <is>
-          <t>86891.76</t>
+          <t>114235</t>
         </is>
       </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
         <is>
-          <t>9318889</t>
+          <t>9318890</t>
         </is>
       </c>
       <c r="B575" s="2" t="inlineStr">
         <is>
-          <t>3232</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C575" s="2" t="inlineStr">
@@ -50385,37 +50385,37 @@
       </c>
       <c r="D575" s="2" t="inlineStr">
         <is>
-          <t>CASA ESPIRITA DO SAMARITANO</t>
+          <t>PM PRESIDENTE KUBITSCHEK</t>
         </is>
       </c>
       <c r="E575" s="2" t="inlineStr">
         <is>
-          <t>01.320.148/0001-76</t>
+          <t>17.754.185/0001-22</t>
         </is>
       </c>
       <c r="F575" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>FEI</t>
         </is>
       </c>
       <c r="G575" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>4601</t>
         </is>
       </c>
       <c r="H575" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>FUNDO ESTADUAL DOS DIREITOS DO IDOSO</t>
         </is>
       </c>
       <c r="I575" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>41</t>
         </is>
       </c>
       <c r="J575" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>CONTRIBUICOES</t>
         </is>
       </c>
       <c r="K575" s="2" t="inlineStr">
@@ -50425,22 +50425,22 @@
       </c>
       <c r="L575" s="2" t="inlineStr">
         <is>
-          <t>SUBVENCOES SOCIAIS</t>
+          <t>CONTRIBUICOES</t>
         </is>
       </c>
       <c r="M575" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>45</t>
         </is>
       </c>
       <c r="N575" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>DOACOES DE PESSOAS, DE INSTITUICOES PRIVADAS OU DO EXTERIOR A ORGAO E ENTIDADES DO ESTADO</t>
         </is>
       </c>
       <c r="O575" s="2" t="inlineStr">
         <is>
-          <t>114235</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="P575" s="2" t="inlineStr">
@@ -50450,19 +50450,19 @@
       </c>
       <c r="Q575" s="2" t="inlineStr">
         <is>
-          <t>114235</t>
+          <t>40000</t>
         </is>
       </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
         <is>
-          <t>9318890</t>
+          <t>9318891</t>
         </is>
       </c>
       <c r="B576" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>3231</t>
         </is>
       </c>
       <c r="C576" s="2" t="inlineStr">
@@ -50472,37 +50472,37 @@
       </c>
       <c r="D576" s="2" t="inlineStr">
         <is>
-          <t>PM PRESIDENTE KUBITSCHEK</t>
+          <t>ASSOC BENEF 08 DE SETEMBRO ASILO STO ANTONIO LAR STO ANTONIO</t>
         </is>
       </c>
       <c r="E576" s="2" t="inlineStr">
         <is>
-          <t>17.754.185/0001-22</t>
+          <t>17.776.188/0001-67</t>
         </is>
       </c>
       <c r="F576" s="2" t="inlineStr">
         <is>
-          <t>FEI</t>
+          <t>FEAS</t>
         </is>
       </c>
       <c r="G576" s="2" t="inlineStr">
         <is>
-          <t>4601</t>
+          <t>4251</t>
         </is>
       </c>
       <c r="H576" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DOS DIREITOS DO IDOSO</t>
+          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
         </is>
       </c>
       <c r="I576" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>43</t>
         </is>
       </c>
       <c r="J576" s="2" t="inlineStr">
         <is>
-          <t>CONTRIBUICOES</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="K576" s="2" t="inlineStr">
@@ -50512,22 +50512,22 @@
       </c>
       <c r="L576" s="2" t="inlineStr">
         <is>
-          <t>CONTRIBUICOES</t>
+          <t>SUBVENCOES SOCIAIS</t>
         </is>
       </c>
       <c r="M576" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>60</t>
         </is>
       </c>
       <c r="N576" s="2" t="inlineStr">
         <is>
-          <t>DOACOES DE PESSOAS, DE INSTITUICOES PRIVADAS OU DO EXTERIOR A ORGAO E ENTIDADES DO ESTADO</t>
+          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
         </is>
       </c>
       <c r="O576" s="2" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>114975.75</t>
         </is>
       </c>
       <c r="P576" s="2" t="inlineStr">
@@ -50537,19 +50537,19 @@
       </c>
       <c r="Q576" s="2" t="inlineStr">
         <is>
-          <t>40000</t>
+          <t>114975.75</t>
         </is>
       </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
         <is>
-          <t>9318891</t>
+          <t>9318892</t>
         </is>
       </c>
       <c r="B577" s="2" t="inlineStr">
         <is>
-          <t>3231</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C577" s="2" t="inlineStr">
@@ -50559,27 +50559,27 @@
       </c>
       <c r="D577" s="2" t="inlineStr">
         <is>
-          <t>ASSOC BENEF 08 DE SETEMBRO ASILO STO ANTONIO LAR STO ANTONIO</t>
+          <t>CARITAS BRASILEIRA</t>
         </is>
       </c>
       <c r="E577" s="2" t="inlineStr">
         <is>
-          <t>17.776.188/0001-67</t>
+          <t>33.654.419/0008-92</t>
         </is>
       </c>
       <c r="F577" s="2" t="inlineStr">
         <is>
-          <t>FEAS</t>
+          <t>SEDESE</t>
         </is>
       </c>
       <c r="G577" s="2" t="inlineStr">
         <is>
-          <t>4251</t>
+          <t>1481</t>
         </is>
       </c>
       <c r="H577" s="2" t="inlineStr">
         <is>
-          <t>FUNDO ESTADUAL DE ASSISTENCIA SOCIAL</t>
+          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
         </is>
       </c>
       <c r="I577" s="2" t="inlineStr">
@@ -50604,17 +50604,17 @@
       </c>
       <c r="M577" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N577" s="2" t="inlineStr">
         <is>
-          <t>RECURSOS DIRETAMENTE ARRECADADOS</t>
+          <t>RECURSOS ORDINARIOS</t>
         </is>
       </c>
       <c r="O577" s="2" t="inlineStr">
         <is>
-          <t>114975.75</t>
+          <t>0</t>
         </is>
       </c>
       <c r="P577" s="2" t="inlineStr">
@@ -50623,93 +50623,6 @@
         </is>
       </c>
       <c r="Q577" s="2" t="inlineStr">
-        <is>
-          <t>114975.75</t>
-        </is>
-      </c>
-    </row>
-    <row r="578">
-      <c r="A578" s="2" t="inlineStr">
-        <is>
-          <t>9318892</t>
-        </is>
-      </c>
-      <c r="B578" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C578" s="2" t="inlineStr">
-        <is>
-          <t>2021-12-30 00:00:00</t>
-        </is>
-      </c>
-      <c r="D578" s="2" t="inlineStr">
-        <is>
-          <t>CARITAS BRASILEIRA</t>
-        </is>
-      </c>
-      <c r="E578" s="2" t="inlineStr">
-        <is>
-          <t>33.654.419/0008-92</t>
-        </is>
-      </c>
-      <c r="F578" s="2" t="inlineStr">
-        <is>
-          <t>SEDESE</t>
-        </is>
-      </c>
-      <c r="G578" s="2" t="inlineStr">
-        <is>
-          <t>1481</t>
-        </is>
-      </c>
-      <c r="H578" s="2" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO SOCIAL</t>
-        </is>
-      </c>
-      <c r="I578" s="2" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="J578" s="2" t="inlineStr">
-        <is>
-          <t>SUBVENCOES SOCIAIS</t>
-        </is>
-      </c>
-      <c r="K578" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="L578" s="2" t="inlineStr">
-        <is>
-          <t>SUBVENCOES SOCIAIS</t>
-        </is>
-      </c>
-      <c r="M578" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="N578" s="2" t="inlineStr">
-        <is>
-          <t>RECURSOS ORDINARIOS</t>
-        </is>
-      </c>
-      <c r="O578" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P578" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="Q578" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>

</xml_diff>